<commit_message>
update no texto 7452
</commit_message>
<xml_diff>
--- a/TEMPLATES/integracao.xlsx
+++ b/TEMPLATES/integracao.xlsx
@@ -9,26 +9,24 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="dados" sheetId="1" r:id="rId1"/>
-    <sheet name="valores" sheetId="3" r:id="rId2"/>
-    <sheet name="propietarios" sheetId="2" r:id="rId3"/>
-    <sheet name="imovel" sheetId="4" r:id="rId4"/>
-    <sheet name="quadro_resumo" sheetId="5" r:id="rId5"/>
-    <sheet name="DECLIVIDADE E PEDOLOGIA" sheetId="6" r:id="rId6"/>
-    <sheet name="respostas" sheetId="7" r:id="rId7"/>
+    <sheet name="propietarios" sheetId="2" r:id="rId2"/>
+    <sheet name="quadro_resumo" sheetId="3" r:id="rId3"/>
+    <sheet name="DECLIVIDADE E PEDOLOGIA" sheetId="4" r:id="rId4"/>
+    <sheet name="respostas" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_Hlk173855386" localSheetId="4">quadro_resumo!$A$1</definedName>
+    <definedName name="_Hlk173855386" localSheetId="2">quadro_resumo!$A$1</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="154">
   <si>
     <t>proponente</t>
   </si>
@@ -54,132 +52,132 @@
     <t>porto nacional - TO</t>
   </si>
   <si>
-    <t>proponente e propietario iguais?</t>
+    <t>mais de um propietario?</t>
+  </si>
+  <si>
+    <t>data de solicitação</t>
+  </si>
+  <si>
+    <t>propietario</t>
+  </si>
+  <si>
+    <t>miguel phelipe feitosa</t>
+  </si>
+  <si>
+    <t>municipio do cartorio</t>
+  </si>
+  <si>
+    <t>palmas - to</t>
+  </si>
+  <si>
+    <t>713.254.791-79</t>
+  </si>
+  <si>
+    <t>data de emissão do cartorio</t>
+  </si>
+  <si>
+    <t>mais de uma matricula?</t>
+  </si>
+  <si>
+    <t>nome do imovel</t>
+  </si>
+  <si>
+    <t>fazenda rancho diamante</t>
+  </si>
+  <si>
+    <t>data da vistoria</t>
+  </si>
+  <si>
+    <t>matricula</t>
+  </si>
+  <si>
+    <t>genero do propietario</t>
+  </si>
+  <si>
+    <t>empresa</t>
+  </si>
+  <si>
+    <t>identificação</t>
+  </si>
+  <si>
+    <t>fazenda</t>
+  </si>
+  <si>
+    <t>casado(a)</t>
+  </si>
+  <si>
+    <t>não</t>
+  </si>
+  <si>
+    <t>area há</t>
+  </si>
+  <si>
+    <t>genero</t>
+  </si>
+  <si>
+    <t>Sr.</t>
+  </si>
+  <si>
+    <t>area construida</t>
+  </si>
+  <si>
+    <t>nome</t>
+  </si>
+  <si>
+    <t>valor de mercado</t>
+  </si>
+  <si>
+    <t>cpf</t>
+  </si>
+  <si>
+    <t>liquidação forçada</t>
+  </si>
+  <si>
+    <t>car</t>
+  </si>
+  <si>
+    <t>TO-1718204-E7A1.2B1B.6B15.4E03.89DD.7006.7298.400E</t>
+  </si>
+  <si>
+    <t>gel</t>
+  </si>
+  <si>
+    <t>c8bdfa60-64a7-4baa-83aa-d84b73759e3e</t>
+  </si>
+  <si>
+    <t>area1</t>
+  </si>
+  <si>
+    <t>area2</t>
+  </si>
+  <si>
+    <t>municipio</t>
+  </si>
+  <si>
+    <t>palmas</t>
+  </si>
+  <si>
+    <t>estado(uf)</t>
+  </si>
+  <si>
+    <t>TO</t>
+  </si>
+  <si>
+    <t>fluid</t>
+  </si>
+  <si>
+    <t>georeferenciamento</t>
+  </si>
+  <si>
+    <t>CAR e Memorial</t>
+  </si>
+  <si>
+    <t>possui hipotecas pendentes?</t>
   </si>
   <si>
     <t>sim</t>
   </si>
   <si>
-    <t>data de solicitação</t>
-  </si>
-  <si>
-    <t>propietario</t>
-  </si>
-  <si>
-    <t>miguel phelipe feitosa</t>
-  </si>
-  <si>
-    <t>municipio do cartorio</t>
-  </si>
-  <si>
-    <t>palmas - to</t>
-  </si>
-  <si>
-    <t>713.254.791-79</t>
-  </si>
-  <si>
-    <t>data de emissão do cartorio</t>
-  </si>
-  <si>
-    <t>mais de um propietario?</t>
-  </si>
-  <si>
-    <t>nome do imovel</t>
-  </si>
-  <si>
-    <t>fazenda rancho diamante</t>
-  </si>
-  <si>
-    <t>data da vistoria</t>
-  </si>
-  <si>
-    <t>matricula</t>
-  </si>
-  <si>
-    <t>genero do propietario</t>
-  </si>
-  <si>
-    <t>empresa</t>
-  </si>
-  <si>
-    <t>identificação</t>
-  </si>
-  <si>
-    <t>fazenda</t>
-  </si>
-  <si>
-    <t>casado(a)</t>
-  </si>
-  <si>
-    <t>não</t>
-  </si>
-  <si>
-    <t>area há</t>
-  </si>
-  <si>
-    <t>genero</t>
-  </si>
-  <si>
-    <t>Sr.</t>
-  </si>
-  <si>
-    <t>area construida</t>
-  </si>
-  <si>
-    <t>nome</t>
-  </si>
-  <si>
-    <t>valor de mercado</t>
-  </si>
-  <si>
-    <t>cpf</t>
-  </si>
-  <si>
-    <t>liquidação forçada</t>
-  </si>
-  <si>
-    <t>car</t>
-  </si>
-  <si>
-    <t>TO-1718204-E7A1.2B1B.6B15.4E03.89DD.7006.7298.400E</t>
-  </si>
-  <si>
-    <t>gel</t>
-  </si>
-  <si>
-    <t>c8bdfa60-64a7-4baa-83aa-d84b73759e3e</t>
-  </si>
-  <si>
-    <t>area1</t>
-  </si>
-  <si>
-    <t>area2</t>
-  </si>
-  <si>
-    <t>municipio</t>
-  </si>
-  <si>
-    <t>palmas</t>
-  </si>
-  <si>
-    <t>estado(uf)</t>
-  </si>
-  <si>
-    <t>TO</t>
-  </si>
-  <si>
-    <t>fluid</t>
-  </si>
-  <si>
-    <t>georeferenciamento</t>
-  </si>
-  <si>
-    <t>CAR e Memorial</t>
-  </si>
-  <si>
-    <t>possuir hipotecas pendentes?</t>
-  </si>
-  <si>
     <t>dentro do bioma amazonico?</t>
   </si>
   <si>
@@ -219,6 +217,9 @@
     <t>liquidação</t>
   </si>
   <si>
+    <t>CODIGO GEL</t>
+  </si>
+  <si>
     <t>propietario 1</t>
   </si>
   <si>
@@ -294,46 +295,13 @@
     <t>matricula10</t>
   </si>
   <si>
-    <t>IMÓVEL</t>
-  </si>
-  <si>
-    <t>Nº Matrícula</t>
-  </si>
-  <si>
-    <t>Valor de mercado</t>
-  </si>
-  <si>
-    <t>Liquidação forçada</t>
-  </si>
-  <si>
-    <t>Identificação</t>
-  </si>
-  <si>
-    <t>Área há</t>
-  </si>
-  <si>
-    <t>Área Construída m²</t>
-  </si>
-  <si>
     <t>QUADRO RESUMO DA AVALIAÇÃO</t>
   </si>
   <si>
-    <t>Agencia:</t>
-  </si>
-  <si>
-    <t>#agencia</t>
-  </si>
-  <si>
     <t>Proponente:</t>
   </si>
   <si>
-    <t>#486: 513.254.791-79</t>
-  </si>
-  <si>
-    <t>Identificação:</t>
-  </si>
-  <si>
-    <t>#nome_imovel</t>
+    <t xml:space="preserve">#486: </t>
   </si>
   <si>
     <t>DECLIVIDADE</t>
@@ -529,7 +497,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -589,8 +557,15 @@
       <name val="Century Gothic"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -699,12 +674,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="17">
     <border>
@@ -902,7 +871,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
@@ -985,47 +954,27 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1352,15 +1301,13 @@
       </c>
     </row>
     <row r="4" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="C4" s="5"/>
       <c r="D4" s="1"/>
       <c r="E4" s="33" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F4" s="8">
         <v>38323</v>
@@ -1368,16 +1315,16 @@
     </row>
     <row r="5" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="E5" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="F5" s="56" t="s">
         <v>13</v>
-      </c>
-      <c r="F5" s="56" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1385,30 +1332,30 @@
         <v>4</v>
       </c>
       <c r="C6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="26" t="s">
         <v>15</v>
-      </c>
-      <c r="E6" s="26" t="s">
-        <v>16</v>
       </c>
       <c r="F6" s="4">
         <v>43822</v>
       </c>
     </row>
     <row r="7" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="50" t="s">
-        <v>17</v>
+      <c r="B7" s="62" t="s">
+        <v>16</v>
       </c>
       <c r="C7" s="5"/>
     </row>
     <row r="8" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="E8" s="27" t="s">
         <v>19</v>
-      </c>
-      <c r="E8" s="27" t="s">
-        <v>20</v>
       </c>
       <c r="F8" s="4">
         <v>42911</v>
@@ -1416,73 +1363,73 @@
     </row>
     <row r="9" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="5">
         <v>1456.6547</v>
       </c>
       <c r="E9" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="38" t="s">
         <v>22</v>
-      </c>
-      <c r="F9" s="38" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="28" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="E10" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="35" t="s">
+      <c r="F10" s="37" t="s">
         <v>26</v>
-      </c>
-      <c r="F10" s="37" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="28" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" s="5">
         <v>1234.5123000000001</v>
       </c>
       <c r="E11" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="39" t="s">
         <v>29</v>
-      </c>
-      <c r="F11" s="39" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" s="5">
         <v>156.65</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F12" s="54"/>
     </row>
     <row r="13" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" s="7">
         <v>25000000</v>
       </c>
       <c r="E13" s="36" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C14" s="7">
         <v>65000000</v>
@@ -1490,23 +1437,23 @@
     </row>
     <row r="15" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C17" s="5">
         <v>100.5205</v>
@@ -1514,7 +1461,7 @@
     </row>
     <row r="18" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C18" s="5">
         <v>321.56479999999999</v>
@@ -1522,23 +1469,23 @@
     </row>
     <row r="19" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="28" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>42</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C21" s="5">
         <v>123456</v>
@@ -1546,18 +1493,18 @@
     </row>
     <row r="22" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>47</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="28" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="29" t="s">
         <v>49</v>
-      </c>
-      <c r="C23" s="29" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1565,7 +1512,7 @@
         <v>50</v>
       </c>
       <c r="C24" s="30" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1612,63 +1559,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-    </row>
-    <row r="2" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="69" t="s">
-        <v>89</v>
-      </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="59"/>
-      <c r="F2" s="69" t="s">
-        <v>90</v>
-      </c>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="59"/>
-      <c r="J2" s="59"/>
-      <c r="K2" s="69" t="s">
-        <v>91</v>
-      </c>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="59"/>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:L23"/>
+  <dimension ref="B1:M24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.28515625" style="63" customWidth="1"/>
@@ -1679,95 +1570,93 @@
     <col min="7" max="8" width="18.7109375" style="63" customWidth="1"/>
     <col min="9" max="9" width="15.85546875" style="63" customWidth="1"/>
     <col min="10" max="10" width="20.5703125" style="63" customWidth="1"/>
-    <col min="11" max="11" width="18.140625" style="63" customWidth="1"/>
-    <col min="12" max="12" width="18.28515625" style="63" customWidth="1"/>
+    <col min="11" max="12" width="18.140625" style="63" customWidth="1"/>
+    <col min="13" max="13" width="18.28515625" style="63" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C2" s="61" t="s">
+    <row r="1" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="59" t="s">
         <v>55</v>
       </c>
-      <c r="D2" s="61" t="s">
+      <c r="D2" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="G2" s="62" t="s">
+      <c r="G2" s="60" t="s">
         <v>57</v>
       </c>
-      <c r="H2" s="62" t="s">
+      <c r="H2" s="60" t="s">
         <v>58</v>
       </c>
-      <c r="I2" s="62" t="s">
+      <c r="I2" s="60" t="s">
         <v>59</v>
       </c>
-      <c r="J2" s="62" t="s">
+      <c r="J2" s="60" t="s">
         <v>60</v>
       </c>
-      <c r="K2" s="62" t="s">
+      <c r="K2" s="60" t="s">
         <v>61</v>
       </c>
-      <c r="L2" s="62" t="s">
+      <c r="L2" s="60" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="3" spans="2:12" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M2" s="60" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="56" t="s">
-        <v>63</v>
-      </c>
-      <c r="C3" s="56" t="str">
-        <f>dados!C5</f>
-        <v>miguel phelipe feitosa</v>
-      </c>
-      <c r="D3" s="55" t="str">
-        <f>dados!C6</f>
-        <v>713.254.791-79</v>
+        <v>64</v>
+      </c>
+      <c r="C3" s="56" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="55" t="s">
+        <v>14</v>
       </c>
       <c r="F3" s="56" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G3" s="56">
-        <f>dados!C9</f>
         <v>1456.6547</v>
       </c>
-      <c r="H3" s="56" t="str">
-        <f>dados!C10</f>
-        <v>fazenda</v>
+      <c r="H3" s="56" t="s">
+        <v>24</v>
       </c>
       <c r="I3" s="56">
-        <f>dados!C11</f>
         <v>1234.5123000000001</v>
       </c>
       <c r="J3" s="56">
-        <f>dados!C12</f>
         <v>156.65</v>
       </c>
-      <c r="K3" s="60">
-        <f>dados!C13</f>
+      <c r="K3" s="58">
         <v>25000000</v>
       </c>
-      <c r="L3" s="60">
-        <f>dados!C14</f>
+      <c r="L3" s="58">
         <v>65000000</v>
       </c>
-    </row>
-    <row r="4" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M3" s="58" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="47" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C4" s="56" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>5</v>
       </c>
       <c r="F4" s="44" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G4" s="47">
         <v>184.096</v>
       </c>
       <c r="H4" s="47" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I4" s="47">
         <v>123.0921</v>
@@ -1781,31 +1670,32 @@
       <c r="L4" s="47">
         <v>1000</v>
       </c>
-    </row>
-    <row r="5" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M4" s="47"/>
+    </row>
+    <row r="5" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="47" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D5" s="47">
         <v>58744</v>
       </c>
       <c r="F5" s="57" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G5" s="56" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H5" s="47" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I5" s="56" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J5" s="56" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K5" s="56">
         <v>10000</v>
@@ -1813,15 +1703,16 @@
       <c r="L5" s="56">
         <v>20000</v>
       </c>
-    </row>
-    <row r="6" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M5" s="56"/>
+    </row>
+    <row r="6" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="47" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="47"/>
       <c r="F6" s="57" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G6" s="56"/>
       <c r="H6" s="56"/>
@@ -1829,15 +1720,16 @@
       <c r="J6" s="56"/>
       <c r="K6" s="56"/>
       <c r="L6" s="56"/>
-    </row>
-    <row r="7" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M6" s="56"/>
+    </row>
+    <row r="7" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="47" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="47"/>
       <c r="F7" s="57" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G7" s="56"/>
       <c r="H7" s="56"/>
@@ -1845,15 +1737,16 @@
       <c r="J7" s="56"/>
       <c r="K7" s="56"/>
       <c r="L7" s="56"/>
-    </row>
-    <row r="8" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M7" s="56"/>
+    </row>
+    <row r="8" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="47" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C8" s="44"/>
       <c r="D8" s="47"/>
       <c r="F8" s="57" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G8" s="56"/>
       <c r="H8" s="56"/>
@@ -1861,14 +1754,15 @@
       <c r="J8" s="56"/>
       <c r="K8" s="56"/>
       <c r="L8" s="56"/>
-    </row>
-    <row r="9" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M8" s="56"/>
+    </row>
+    <row r="9" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="46" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D9" s="47"/>
       <c r="F9" s="57" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G9" s="56"/>
       <c r="H9" s="56"/>
@@ -1876,15 +1770,16 @@
       <c r="J9" s="56"/>
       <c r="K9" s="56"/>
       <c r="L9" s="56"/>
-    </row>
-    <row r="10" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M9" s="56"/>
+    </row>
+    <row r="10" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="56" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C10" s="53"/>
       <c r="D10" s="47"/>
       <c r="F10" s="57" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G10" s="56"/>
       <c r="H10" s="56"/>
@@ -1892,15 +1787,16 @@
       <c r="J10" s="56"/>
       <c r="K10" s="56"/>
       <c r="L10" s="56"/>
-    </row>
-    <row r="11" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M10" s="56"/>
+    </row>
+    <row r="11" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="45" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C11" s="51"/>
       <c r="D11" s="47"/>
       <c r="F11" s="57" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G11" s="56"/>
       <c r="H11" s="56"/>
@@ -1908,15 +1804,16 @@
       <c r="J11" s="56"/>
       <c r="K11" s="56"/>
       <c r="L11" s="56"/>
-    </row>
-    <row r="12" spans="2:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M11" s="56"/>
+    </row>
+    <row r="12" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="56" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C12" s="53"/>
       <c r="D12" s="47"/>
       <c r="F12" s="57" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G12" s="56"/>
       <c r="H12" s="56"/>
@@ -1924,18 +1821,79 @@
       <c r="J12" s="56"/>
       <c r="K12" s="56"/>
       <c r="L12" s="56"/>
-    </row>
-    <row r="13" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="2:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="M12" s="56"/>
+    </row>
+    <row r="13" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="59" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="59" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" s="59" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="56" t="str">
+        <f>dados!F11</f>
+        <v>Sr.</v>
+      </c>
+      <c r="C15" s="56">
+        <f>dados!F12</f>
+        <v>0</v>
+      </c>
+      <c r="D15" s="56">
+        <f>dados!F13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="56"/>
+      <c r="C16" s="56"/>
+      <c r="D16" s="56"/>
+    </row>
+    <row r="17" spans="2:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="56"/>
+      <c r="C17" s="56"/>
+      <c r="D17" s="56"/>
+    </row>
+    <row r="18" spans="2:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="56"/>
+      <c r="C18" s="56"/>
+      <c r="D18" s="56"/>
+    </row>
+    <row r="19" spans="2:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="56"/>
+      <c r="C19" s="56"/>
+      <c r="D19" s="56"/>
+    </row>
+    <row r="20" spans="2:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="56"/>
+      <c r="C20" s="56"/>
+      <c r="D20" s="56"/>
+    </row>
+    <row r="21" spans="2:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="56"/>
+      <c r="C21" s="56"/>
+      <c r="D21" s="56"/>
+    </row>
+    <row r="22" spans="2:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="56"/>
+      <c r="C22" s="56"/>
+      <c r="D22" s="56"/>
+    </row>
+    <row r="23" spans="2:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="56"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="56"/>
+    </row>
+    <row r="24" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="56"/>
+      <c r="C24" s="56"/>
+      <c r="D24" s="56"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="deixe no formata de cpf ou cnpj ಠ‿ಠ_x000a__x000a_000.000.000-00_x000a__x000a_00.000.000/0000-00" sqref="D4"/>
@@ -1945,166 +1903,77 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="14" width="9.140625" style="64" customWidth="1"/>
+    <col min="1" max="63" width="9.140625" style="63" customWidth="1"/>
+    <col min="64" max="16384" width="9.140625" style="63"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="69" t="s">
+    <row r="1" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="69" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="69" t="s">
-        <v>92</v>
-      </c>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="69" t="s">
-        <v>93</v>
-      </c>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="69" t="s">
-        <v>94</v>
-      </c>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="58"/>
+      <c r="B1" s="66"/>
+      <c r="C1" s="66"/>
+      <c r="D1" s="66"/>
+      <c r="E1" s="66"/>
+      <c r="F1" s="66"/>
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+      <c r="M1" s="66"/>
+      <c r="N1" s="66"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="66"/>
+      <c r="Q1" s="66"/>
+      <c r="R1" s="66"/>
+      <c r="S1" s="66"/>
+    </row>
+    <row r="2" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="65" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="66"/>
+      <c r="C2" s="67" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="61" t="s">
+        <v>91</v>
+      </c>
+      <c r="K2" s="68" t="s">
+        <v>5</v>
+      </c>
+      <c r="L2" s="66"/>
+      <c r="M2" s="66"/>
+      <c r="N2" s="66"/>
+      <c r="O2" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="O1:S1"/>
+    <mergeCell ref="C2:I2"/>
+    <mergeCell ref="K2:N2"/>
     <mergeCell ref="A1:N1"/>
-    <mergeCell ref="J2:M2"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="G2:I2"/>
-  </mergeCells>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="61" width="9.140625" style="63" customWidth="1"/>
-    <col min="62" max="16384" width="9.140625" style="63"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="73" t="s">
-        <v>95</v>
-      </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="74" t="s">
-        <v>96</v>
-      </c>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="71" t="s">
-        <v>97</v>
-      </c>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="68"/>
-      <c r="U1" s="68"/>
-      <c r="V1" s="68"/>
-      <c r="W1" s="68"/>
-      <c r="X1" s="71"/>
-      <c r="Y1" s="68"/>
-      <c r="Z1" s="68"/>
-      <c r="AA1" s="68"/>
-      <c r="AB1" s="68"/>
-    </row>
-    <row r="2" spans="1:28" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="74" t="s">
-        <v>98</v>
-      </c>
-      <c r="B2" s="68"/>
-      <c r="C2" s="71" t="str">
-        <f>dados!C2</f>
-        <v>marco antonio feitosa</v>
-      </c>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="72" t="s">
-        <v>99</v>
-      </c>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="65" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q2" s="75" t="s">
-        <v>101</v>
-      </c>
-      <c r="R2" s="68"/>
-      <c r="S2" s="68"/>
-      <c r="T2" s="68"/>
-      <c r="U2" s="68"/>
-      <c r="V2" s="68"/>
-      <c r="W2" s="68"/>
-      <c r="X2" s="66"/>
-    </row>
-  </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="X1:AB1"/>
-    <mergeCell ref="J2:N2"/>
-    <mergeCell ref="C2:I2"/>
-    <mergeCell ref="Q1:W1"/>
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="O1:P1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="Q2:W2"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:C33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2116,227 +1985,227 @@
     <row r="1" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="19" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="C2" s="54" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="14" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="13" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="13" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="56" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="C13" s="56" t="s">
-        <v>103</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="16" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="16" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="17" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="17" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="17" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="17" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="17" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="16" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="16" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="16" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="17" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="17" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="16" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="17" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="17" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="16" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="16" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="16" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="17" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
     </row>
     <row r="33" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="16" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -2344,7 +2213,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Planilha2"/>
   <dimension ref="A1:D5"/>
@@ -2358,58 +2227,58 @@
   <sheetData>
     <row r="1" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="40" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="B1" s="41" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C1" s="41" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="D1" s="42" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="43" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="43" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B3" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="43" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" s="1"/>
     </row>
     <row r="5" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="44" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>

</xml_diff>

<commit_message>
fazendo o quadro de amostras
</commit_message>
<xml_diff>
--- a/TEMPLATES/integracao.xlsx
+++ b/TEMPLATES/integracao.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="EstaPasta_de_trabalho" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\automatizar_descritivo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\automatizar_descritivo\TEMPLATES\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="dados" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="153">
   <si>
     <t>proponente</t>
   </si>
@@ -299,9 +299,6 @@
   </si>
   <si>
     <t>Proponente:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#486: </t>
   </si>
   <si>
     <t>DECLIVIDADE</t>
@@ -497,7 +494,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -553,13 +550,6 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Century Gothic"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
       <family val="2"/>
@@ -957,7 +947,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -970,11 +959,12 @@
     <xf numFmtId="0" fontId="7" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1260,10 +1250,10 @@
   <dimension ref="B1:F29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="31.85546875" style="63" customWidth="1"/>
+    <col min="2" max="2" width="31.85546875" style="62" customWidth="1"/>
     <col min="3" max="3" width="51.5703125" style="52" customWidth="1"/>
-    <col min="5" max="5" width="31.28515625" style="63" customWidth="1"/>
-    <col min="6" max="6" width="21.85546875" style="63" customWidth="1"/>
+    <col min="5" max="5" width="31.28515625" style="62" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" style="62" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1342,7 +1332,7 @@
       </c>
     </row>
     <row r="7" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="62" t="s">
+      <c r="B7" s="61" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="5"/>
@@ -1562,16 +1552,16 @@
   <dimension ref="B1:M24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" style="63" customWidth="1"/>
-    <col min="3" max="3" width="27.7109375" style="63" customWidth="1"/>
-    <col min="4" max="4" width="20" style="63" customWidth="1"/>
-    <col min="5" max="5" width="24.140625" style="63" customWidth="1"/>
-    <col min="6" max="6" width="28.140625" style="63" customWidth="1"/>
-    <col min="7" max="8" width="18.7109375" style="63" customWidth="1"/>
-    <col min="9" max="9" width="15.85546875" style="63" customWidth="1"/>
-    <col min="10" max="10" width="20.5703125" style="63" customWidth="1"/>
-    <col min="11" max="12" width="18.140625" style="63" customWidth="1"/>
-    <col min="13" max="13" width="18.28515625" style="63" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="62" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" style="62" customWidth="1"/>
+    <col min="4" max="4" width="20" style="62" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" style="62" customWidth="1"/>
+    <col min="6" max="6" width="28.140625" style="62" customWidth="1"/>
+    <col min="7" max="8" width="18.7109375" style="62" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" style="62" customWidth="1"/>
+    <col min="10" max="10" width="20.5703125" style="62" customWidth="1"/>
+    <col min="11" max="12" width="18.140625" style="62" customWidth="1"/>
+    <col min="13" max="13" width="18.28515625" style="62" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -1908,65 +1898,64 @@
   <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="63" width="9.140625" style="63" customWidth="1"/>
-    <col min="64" max="16384" width="9.140625" style="63"/>
+    <col min="1" max="63" width="9.140625" style="62" customWidth="1"/>
+    <col min="64" max="16384" width="9.140625" style="62"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="67" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="66"/>
-      <c r="H1" s="66"/>
-      <c r="I1" s="66"/>
-      <c r="J1" s="66"/>
-      <c r="K1" s="66"/>
-      <c r="L1" s="66"/>
-      <c r="M1" s="66"/>
-      <c r="N1" s="66"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="66"/>
-      <c r="Q1" s="66"/>
-      <c r="R1" s="66"/>
-      <c r="S1" s="66"/>
+      <c r="B1" s="65"/>
+      <c r="C1" s="65"/>
+      <c r="D1" s="65"/>
+      <c r="E1" s="65"/>
+      <c r="F1" s="65"/>
+      <c r="G1" s="65"/>
+      <c r="H1" s="65"/>
+      <c r="I1" s="65"/>
+      <c r="J1" s="65"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="65"/>
+      <c r="M1" s="65"/>
+      <c r="N1" s="65"/>
+      <c r="O1" s="66"/>
+      <c r="P1" s="65"/>
+      <c r="Q1" s="65"/>
+      <c r="R1" s="65"/>
+      <c r="S1" s="65"/>
     </row>
     <row r="2" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="64" t="s">
         <v>90</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="67" t="s">
+      <c r="B2" s="65"/>
+      <c r="C2" s="66" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="61" t="s">
-        <v>91</v>
-      </c>
-      <c r="K2" s="68" t="s">
-        <v>5</v>
-      </c>
-      <c r="L2" s="66"/>
-      <c r="M2" s="66"/>
-      <c r="N2" s="66"/>
-      <c r="O2" s="64"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="65"/>
+      <c r="I2" s="65"/>
+      <c r="J2" s="69" t="str">
+        <f>"486: " &amp; dados!C3</f>
+        <v>486: 32.251.489/5614-55</v>
+      </c>
+      <c r="K2" s="69"/>
+      <c r="L2" s="69"/>
+      <c r="M2" s="69"/>
+      <c r="N2" s="68"/>
+      <c r="O2" s="63"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="O1:S1"/>
     <mergeCell ref="C2:I2"/>
-    <mergeCell ref="K2:N2"/>
     <mergeCell ref="A1:N1"/>
+    <mergeCell ref="J2:M2"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1978,234 +1967,234 @@
   <dimension ref="B1:C33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="61" style="63" customWidth="1"/>
-    <col min="3" max="3" width="90.85546875" style="63" customWidth="1"/>
+    <col min="2" max="2" width="61" style="62" customWidth="1"/>
+    <col min="3" max="3" width="90.85546875" style="62" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="54" t="s">
         <v>92</v>
-      </c>
-      <c r="C2" s="54" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="20" t="s">
         <v>94</v>
-      </c>
-      <c r="C3" s="20" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="4" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" s="15" t="s">
         <v>96</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="5" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>98</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="21" t="s">
         <v>100</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="21" t="s">
         <v>102</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" s="21" t="s">
         <v>104</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="2:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B13" s="56" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C13" s="56" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="15" t="s">
         <v>107</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="15" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>109</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="C16" s="15" t="s">
         <v>111</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" s="15" t="s">
         <v>113</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="17" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" s="15" t="s">
         <v>115</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" s="15" t="s">
         <v>117</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="C20" s="15" t="s">
         <v>119</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="C21" s="18" t="s">
         <v>121</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="16" t="s">
+        <v>122</v>
+      </c>
+      <c r="C22" s="18" t="s">
         <v>123</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="C23" s="18" t="s">
         <v>125</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="C24" s="18" t="s">
         <v>127</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="25" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="C25" s="15" t="s">
         <v>129</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="C26" s="15" t="s">
         <v>131</v>
-      </c>
-      <c r="C26" s="15" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="C27" s="15" t="s">
         <v>133</v>
-      </c>
-      <c r="C27" s="15" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="C28" s="15" t="s">
         <v>135</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="16" t="s">
+        <v>136</v>
+      </c>
+      <c r="C29" s="15" t="s">
         <v>137</v>
-      </c>
-      <c r="C29" s="15" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B30" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="C30" s="15" t="s">
         <v>139</v>
-      </c>
-      <c r="C30" s="15" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="C31" s="15" t="s">
         <v>141</v>
-      </c>
-      <c r="C31" s="15" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="32" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="C32" s="15" t="s">
         <v>143</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="33" spans="2:3" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="C33" s="15" t="s">
         <v>145</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -2219,29 +2208,29 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" style="63" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" style="63" customWidth="1"/>
-    <col min="3" max="3" width="14" style="63" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" style="63" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" style="62" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" style="62" customWidth="1"/>
+    <col min="3" max="3" width="14" style="62" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" style="62" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="40" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B1" s="41" t="s">
         <v>21</v>
       </c>
       <c r="C1" s="41" t="s">
+        <v>147</v>
+      </c>
+      <c r="D1" s="42" t="s">
         <v>148</v>
-      </c>
-      <c r="D1" s="42" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="43" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B2" t="s">
         <v>29</v>
@@ -2255,10 +2244,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="43" t="s">
+        <v>150</v>
+      </c>
+      <c r="B3" t="s">
         <v>151</v>
-      </c>
-      <c r="B3" t="s">
-        <v>152</v>
       </c>
       <c r="C3" t="s">
         <v>26</v>
@@ -2269,7 +2258,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="43" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B4" t="s">
         <v>22</v>

</xml_diff>